<commit_message>
Fix residential-tips hero, cards, and DM image handling
- hero.css: overlay text on a dark maroon panel over the image at all
  breakpoints (matches source design)
- hero/cards-promo models: image field reference -> richtext so md2jcr
  handles extension-less Dynamic Media URLs
- cards-promo/hero parsers: preserve section headings; bake in lazy-loaded
  accordion bodies; skip optimizer for DM URLs
- xcelenergy-cleanup transformer: strip aura error box, feedback/backtick
  artifacts; rename Xcel -> X in visible text only

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-residential-tips.report.xlsx
+++ b/tools/importer/reports/import-residential-tips.report.xlsx
@@ -52,10 +52,10 @@
     <t>residential-tips</t>
   </si>
   <si>
-    <t>2026-07-30T13:31:15.734Z</t>
-  </si>
-  <si>
-    <t>Energy Saving Tips | Residential Services | Xcel Energy</t>
+    <t>2026-07-31T03:43:39.130Z</t>
+  </si>
+  <si>
+    <t>Energy Saving Tips | Residential Services | X Energy</t>
   </si>
   <si>
     <t>https://co.my.xcelenergy.com/s/residential/tips</t>

</xml_diff>

<commit_message>
Fix residential-tips hero, cards, and Dynamic Media image handling (#9)
- hero.css: overlay text on a dark maroon panel over the image at all
  breakpoints (matches source design)
- hero/cards-promo models: image field reference -> richtext so md2jcr
  handles extension-less Dynamic Media URLs
- cards-promo/hero parsers: preserve section headings; bake in lazy-loaded
  accordion bodies; skip optimizer for DM URLs
- xcelenergy-cleanup transformer: strip aura error box, feedback/backtick
  artifacts; rename Xcel -> X in visible text only

Co-authored-by: AEMY Studio <noreply@aemy.studio>
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-residential-tips.report.xlsx
+++ b/tools/importer/reports/import-residential-tips.report.xlsx
@@ -52,10 +52,10 @@
     <t>residential-tips</t>
   </si>
   <si>
-    <t>2026-07-30T13:31:15.734Z</t>
-  </si>
-  <si>
-    <t>Energy Saving Tips | Residential Services | Xcel Energy</t>
+    <t>2026-07-31T03:43:39.130Z</t>
+  </si>
+  <si>
+    <t>Energy Saving Tips | Residential Services | X Energy</t>
   </si>
   <si>
     <t>https://co.my.xcelenergy.com/s/residential/tips</t>

</xml_diff>